<commit_message>
Update MOM Excel template
</commit_message>
<xml_diff>
--- a/mom_app/SRMD MOM Format.xlsx
+++ b/mom_app/SRMD MOM Format.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aryanshah/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aryanshah/Desktop/Codex/mom_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A1931A1C-9B02-124F-90AB-41275B5F0B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE707847-8008-6F41-A4C8-8A1D361990E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="660" windowWidth="22820" windowHeight="16540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="660" windowWidth="23920" windowHeight="16540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mom" sheetId="4" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Mom!$B$1:$F$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Mom!$B$1:$F$33</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>MINUTES OF MEETING</t>
   </si>
@@ -72,6 +72,15 @@
   </si>
   <si>
     <t>Discipline of Work</t>
+  </si>
+  <si>
+    <t>Sr No</t>
+  </si>
+  <si>
+    <t>Full Name</t>
+  </si>
+  <si>
+    <t>Agency</t>
   </si>
 </sst>
 </file>
@@ -176,7 +185,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="62">
+  <borders count="61">
     <border>
       <left/>
       <right/>
@@ -298,34 +307,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="medium">
@@ -958,6 +939,17 @@
       </top>
       <bottom style="thin">
         <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -965,30 +957,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1003,44 +980,44 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
@@ -1048,211 +1025,235 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="56" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="42" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="54" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="40" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="50" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="48" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="40" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="39" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="38" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="55" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="57" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="61" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1558,12 +1559,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.5" customWidth="1"/>
     <col min="2" max="2" width="13.5" customWidth="1"/>
-    <col min="3" max="3" width="39.1640625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="39.1640625" style="4" customWidth="1"/>
     <col min="4" max="5" width="30.1640625" customWidth="1"/>
     <col min="6" max="6" width="52.83203125" customWidth="1"/>
     <col min="7" max="7" width="7.5" customWidth="1"/>
@@ -1572,425 +1573,453 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" thickBot="1">
-      <c r="A1" s="39"/>
-      <c r="B1" s="36"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="30"/>
+      <c r="A1" s="34"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="25"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" thickBot="1">
-      <c r="A2" s="40"/>
-      <c r="B2" s="52" t="s">
+      <c r="A2" s="35"/>
+      <c r="B2" s="78" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="30"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="80"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="25"/>
     </row>
     <row r="3" spans="1:8" ht="19" thickBot="1">
-      <c r="A3" s="40"/>
-      <c r="B3" s="55" t="s">
+      <c r="A3" s="35"/>
+      <c r="B3" s="81" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="30"/>
+      <c r="C3" s="82"/>
+      <c r="D3" s="82"/>
+      <c r="E3" s="82"/>
+      <c r="F3" s="83"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="25"/>
     </row>
     <row r="4" spans="1:8" ht="18" thickBot="1">
-      <c r="A4" s="40"/>
-      <c r="B4" s="8" t="s">
+      <c r="A4" s="35"/>
+      <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="93"/>
-      <c r="F4" s="59"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="30"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="84"/>
+      <c r="E4" s="85"/>
+      <c r="F4" s="86"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="25"/>
     </row>
     <row r="5" spans="1:8" ht="18" thickBot="1">
-      <c r="A5" s="40"/>
-      <c r="B5" s="8" t="s">
+      <c r="A5" s="35"/>
+      <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="1"/>
-      <c r="D5" s="60"/>
-      <c r="E5" s="94"/>
-      <c r="F5" s="61"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="30"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="88"/>
+      <c r="F5" s="89"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="25"/>
     </row>
     <row r="6" spans="1:8" ht="18" thickBot="1">
-      <c r="A6" s="40"/>
-      <c r="B6" s="8" t="s">
+      <c r="A6" s="35"/>
+      <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="95"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="30"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="91"/>
+      <c r="F6" s="92"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="25"/>
     </row>
     <row r="7" spans="1:8" ht="16" thickBot="1">
-      <c r="A7" s="40"/>
-      <c r="B7" s="64"/>
-      <c r="C7" s="65"/>
-      <c r="D7" s="65"/>
-      <c r="E7" s="65"/>
-      <c r="F7" s="66"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="30"/>
-    </row>
-    <row r="8" spans="1:8" ht="18" thickBot="1">
-      <c r="A8" s="40"/>
-      <c r="B8" s="2" t="s">
+      <c r="A7" s="35"/>
+      <c r="B7" s="93"/>
+      <c r="C7" s="94"/>
+      <c r="D7" s="94"/>
+      <c r="E7" s="94"/>
+      <c r="F7" s="95"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="25"/>
+    </row>
+    <row r="8" spans="1:8" ht="18" customHeight="1" thickBot="1">
+      <c r="A8" s="35"/>
+      <c r="B8" s="104" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="68"/>
-      <c r="D8" s="69"/>
-      <c r="E8" s="69"/>
-      <c r="F8" s="70"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="30"/>
-    </row>
-    <row r="9" spans="1:8" ht="17" thickBot="1">
-      <c r="A9" s="40"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="73"/>
-      <c r="E9" s="96"/>
-      <c r="F9" s="74"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="30"/>
+      <c r="C8" s="105"/>
+      <c r="D8" s="105"/>
+      <c r="E8" s="105"/>
+      <c r="F8" s="106"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="25"/>
+    </row>
+    <row r="9" spans="1:8" ht="18" customHeight="1" thickBot="1">
+      <c r="A9" s="35"/>
+      <c r="B9" s="107" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="108" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="108" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="102"/>
+      <c r="F9" s="103"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="25"/>
     </row>
     <row r="10" spans="1:8" ht="17" thickBot="1">
-      <c r="A10" s="40"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="73"/>
-      <c r="E10" s="96"/>
-      <c r="F10" s="74"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="30"/>
+      <c r="A10" s="35"/>
+      <c r="B10" s="98">
+        <v>1</v>
+      </c>
+      <c r="C10" s="6"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="25"/>
     </row>
     <row r="11" spans="1:8" ht="17" thickBot="1">
-      <c r="A11" s="40"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="75"/>
-      <c r="E11" s="97"/>
-      <c r="F11" s="76"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="30"/>
+      <c r="A11" s="35"/>
+      <c r="B11" s="98">
+        <v>2</v>
+      </c>
+      <c r="C11" s="6"/>
+      <c r="D11" s="44"/>
+      <c r="E11" s="45"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="25"/>
     </row>
     <row r="12" spans="1:8" ht="17" thickBot="1">
-      <c r="A12" s="40"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="77"/>
-      <c r="E12" s="98"/>
-      <c r="F12" s="78"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="30"/>
+      <c r="A12" s="35"/>
+      <c r="B12" s="99">
+        <v>3</v>
+      </c>
+      <c r="C12" s="7"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="48"/>
+      <c r="F12" s="49"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="25"/>
     </row>
     <row r="13" spans="1:8" ht="17" thickBot="1">
-      <c r="A13" s="40"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="71"/>
-      <c r="E13" s="98"/>
-      <c r="F13" s="72"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="30"/>
+      <c r="A13" s="35"/>
+      <c r="B13" s="100">
+        <v>4</v>
+      </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="50"/>
+      <c r="E13" s="41"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="25"/>
     </row>
     <row r="14" spans="1:8" ht="17" thickBot="1">
-      <c r="A14" s="40"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="71"/>
-      <c r="E14" s="98"/>
-      <c r="F14" s="72"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="30"/>
-    </row>
-    <row r="15" spans="1:8" ht="16" thickBot="1">
-      <c r="A15" s="40"/>
-      <c r="B15" s="79"/>
-      <c r="C15" s="80"/>
-      <c r="D15" s="80"/>
-      <c r="E15" s="99"/>
-      <c r="F15" s="81"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="30"/>
-    </row>
-    <row r="16" spans="1:8" ht="19" thickBot="1">
-      <c r="A16" s="40"/>
-      <c r="B16" s="82" t="s">
+      <c r="A14" s="35"/>
+      <c r="B14" s="101">
         <v>5</v>
       </c>
-      <c r="C16" s="83"/>
-      <c r="D16" s="83"/>
-      <c r="E16" s="100"/>
-      <c r="F16" s="84"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="30"/>
-    </row>
-    <row r="17" spans="1:10" s="18" customFormat="1" ht="21" customHeight="1" thickBot="1">
-      <c r="A17" s="41"/>
-      <c r="B17" s="17" t="s">
+      <c r="C14" s="9"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="41"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="25"/>
+    </row>
+    <row r="15" spans="1:8" ht="17" thickBot="1">
+      <c r="A15" s="35"/>
+      <c r="B15" s="101">
         <v>6</v>
       </c>
-      <c r="C17" s="85" t="s">
+      <c r="C15" s="9"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="42"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="25"/>
+    </row>
+    <row r="16" spans="1:8" ht="16" thickBot="1">
+      <c r="A16" s="35"/>
+      <c r="B16" s="52"/>
+      <c r="C16" s="53"/>
+      <c r="D16" s="53"/>
+      <c r="E16" s="54"/>
+      <c r="F16" s="55"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="25"/>
+    </row>
+    <row r="17" spans="1:10" ht="19" thickBot="1">
+      <c r="A17" s="35"/>
+      <c r="B17" s="56" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="57"/>
+      <c r="D17" s="57"/>
+      <c r="E17" s="58"/>
+      <c r="F17" s="59"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="25"/>
+    </row>
+    <row r="18" spans="1:10" s="13" customFormat="1" ht="21" customHeight="1" thickBot="1">
+      <c r="A18" s="36"/>
+      <c r="B18" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="86"/>
-      <c r="E17" s="101" t="s">
+      <c r="D18" s="61"/>
+      <c r="E18" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="F17" s="23" t="s">
+      <c r="F18" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="28"/>
-      <c r="H17" s="31"/>
-    </row>
-    <row r="18" spans="1:10" ht="31.5" customHeight="1">
-      <c r="A18" s="40"/>
-      <c r="B18" s="15">
+      <c r="G18" s="23"/>
+      <c r="H18" s="26"/>
+    </row>
+    <row r="19" spans="1:10" ht="31.5" customHeight="1">
+      <c r="A19" s="35"/>
+      <c r="B19" s="10">
         <v>1</v>
       </c>
-      <c r="C18" s="45"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="30"/>
-    </row>
-    <row r="19" spans="1:10" ht="33.75" customHeight="1">
-      <c r="A19" s="40"/>
-      <c r="B19" s="16">
+      <c r="C19" s="97"/>
+      <c r="D19" s="97"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="25"/>
+    </row>
+    <row r="20" spans="1:10" ht="33.75" customHeight="1">
+      <c r="A20" s="35"/>
+      <c r="B20" s="11">
         <v>2</v>
       </c>
-      <c r="C19" s="44"/>
-      <c r="D19" s="44"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="30"/>
-      <c r="J19" s="7"/>
-    </row>
-    <row r="20" spans="1:10" ht="47.25" customHeight="1">
-      <c r="A20" s="40"/>
-      <c r="B20" s="16">
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="25"/>
+      <c r="J20" s="2"/>
+    </row>
+    <row r="21" spans="1:10" ht="47.25" customHeight="1">
+      <c r="A21" s="35"/>
+      <c r="B21" s="11">
         <v>3</v>
       </c>
-      <c r="C20" s="44"/>
-      <c r="D20" s="44"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="30"/>
-    </row>
-    <row r="21" spans="1:10" ht="42.75" customHeight="1">
-      <c r="A21" s="40"/>
-      <c r="B21" s="16">
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="25"/>
+    </row>
+    <row r="22" spans="1:10" ht="42.75" customHeight="1">
+      <c r="A22" s="35"/>
+      <c r="B22" s="11">
         <v>4</v>
       </c>
-      <c r="C21" s="44"/>
-      <c r="D21" s="44"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="30"/>
-    </row>
-    <row r="22" spans="1:10" ht="17.25" customHeight="1">
-      <c r="A22" s="40"/>
-      <c r="B22" s="16">
+      <c r="C22" s="43"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="25"/>
+    </row>
+    <row r="23" spans="1:10" ht="17.25" customHeight="1">
+      <c r="A23" s="35"/>
+      <c r="B23" s="11">
         <v>5</v>
       </c>
-      <c r="C22" s="44"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="20"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="30"/>
-    </row>
-    <row r="23" spans="1:10" ht="29.25" customHeight="1">
-      <c r="A23" s="40"/>
-      <c r="B23" s="16">
+      <c r="C23" s="43"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="22"/>
+      <c r="H23" s="25"/>
+    </row>
+    <row r="24" spans="1:10" ht="29.25" customHeight="1">
+      <c r="A24" s="35"/>
+      <c r="B24" s="11">
         <v>6</v>
       </c>
-      <c r="C23" s="44"/>
-      <c r="D23" s="44"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="30"/>
-    </row>
-    <row r="24" spans="1:10" ht="34.5" customHeight="1">
-      <c r="A24" s="40"/>
-      <c r="B24" s="16">
+      <c r="C24" s="43"/>
+      <c r="D24" s="43"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="22"/>
+      <c r="H24" s="25"/>
+    </row>
+    <row r="25" spans="1:10" ht="34.5" customHeight="1">
+      <c r="A25" s="35"/>
+      <c r="B25" s="11">
         <v>7</v>
       </c>
-      <c r="C24" s="44"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="30"/>
-    </row>
-    <row r="25" spans="1:10" ht="17.25" customHeight="1">
-      <c r="A25" s="40"/>
-      <c r="B25" s="16">
+      <c r="C25" s="43"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="25"/>
+    </row>
+    <row r="26" spans="1:10" ht="17.25" customHeight="1">
+      <c r="A26" s="35"/>
+      <c r="B26" s="11">
         <v>8</v>
       </c>
-      <c r="C25" s="44"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="30"/>
-    </row>
-    <row r="26" spans="1:10" ht="17.25" customHeight="1">
-      <c r="A26" s="40"/>
-      <c r="B26" s="16">
+      <c r="C26" s="43"/>
+      <c r="D26" s="43"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="25"/>
+    </row>
+    <row r="27" spans="1:10" ht="17.25" customHeight="1">
+      <c r="A27" s="35"/>
+      <c r="B27" s="11">
         <v>9</v>
       </c>
-      <c r="C26" s="44"/>
-      <c r="D26" s="44"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="27"/>
-      <c r="H26" s="30"/>
-    </row>
-    <row r="27" spans="1:10" ht="17.25" customHeight="1" thickBot="1">
-      <c r="A27" s="40"/>
-      <c r="B27" s="22"/>
       <c r="C27" s="43"/>
       <c r="D27" s="43"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="27"/>
-      <c r="H27" s="30"/>
-    </row>
-    <row r="28" spans="1:10" ht="16" thickBot="1">
-      <c r="A28" s="40"/>
-      <c r="B28" s="49"/>
-      <c r="C28" s="50"/>
-      <c r="D28" s="50"/>
-      <c r="E28" s="103"/>
-      <c r="F28" s="51"/>
-      <c r="G28" s="27"/>
-      <c r="H28" s="30"/>
-    </row>
-    <row r="29" spans="1:10" ht="19.5" customHeight="1" thickBot="1">
-      <c r="A29" s="40"/>
-      <c r="B29" s="87" t="s">
+      <c r="E27" s="15"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="25"/>
+    </row>
+    <row r="28" spans="1:10" ht="17.25" customHeight="1" thickBot="1">
+      <c r="A28" s="35"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="96"/>
+      <c r="D28" s="96"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="25"/>
+    </row>
+    <row r="29" spans="1:10" ht="16" thickBot="1">
+      <c r="A29" s="35"/>
+      <c r="B29" s="74"/>
+      <c r="C29" s="75"/>
+      <c r="D29" s="75"/>
+      <c r="E29" s="76"/>
+      <c r="F29" s="77"/>
+      <c r="G29" s="22"/>
+      <c r="H29" s="25"/>
+    </row>
+    <row r="30" spans="1:10" ht="19.5" customHeight="1" thickBot="1">
+      <c r="A30" s="35"/>
+      <c r="B30" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="C29" s="88"/>
-      <c r="D29" s="88"/>
-      <c r="E29" s="104"/>
-      <c r="F29" s="89"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="30"/>
-    </row>
-    <row r="30" spans="1:10">
-      <c r="A30" s="40"/>
-      <c r="B30" s="46"/>
-      <c r="C30" s="47"/>
-      <c r="D30" s="47"/>
-      <c r="E30" s="102"/>
-      <c r="F30" s="48"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="30"/>
+      <c r="C30" s="63"/>
+      <c r="D30" s="63"/>
+      <c r="E30" s="64"/>
+      <c r="F30" s="65"/>
+      <c r="G30" s="22"/>
+      <c r="H30" s="25"/>
     </row>
     <row r="31" spans="1:10">
-      <c r="A31" s="40"/>
-      <c r="B31" s="90"/>
-      <c r="C31" s="91"/>
-      <c r="D31" s="91"/>
-      <c r="E31" s="105"/>
-      <c r="F31" s="92"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="30"/>
-    </row>
-    <row r="32" spans="1:10" ht="16" thickBot="1">
-      <c r="A32" s="40"/>
-      <c r="B32" s="49"/>
-      <c r="C32" s="50"/>
-      <c r="D32" s="50"/>
-      <c r="E32" s="103"/>
-      <c r="F32" s="51"/>
-      <c r="G32" s="27"/>
-      <c r="H32" s="30"/>
-    </row>
-    <row r="33" spans="1:8" ht="30" customHeight="1">
-      <c r="A33" s="40"/>
-      <c r="B33" s="27"/>
-      <c r="C33" s="67" t="str">
-        <f>UPPER(C32)</f>
+      <c r="A31" s="35"/>
+      <c r="B31" s="66"/>
+      <c r="C31" s="67"/>
+      <c r="D31" s="67"/>
+      <c r="E31" s="68"/>
+      <c r="F31" s="69"/>
+      <c r="G31" s="22"/>
+      <c r="H31" s="25"/>
+    </row>
+    <row r="32" spans="1:10">
+      <c r="A32" s="35"/>
+      <c r="B32" s="70"/>
+      <c r="C32" s="71"/>
+      <c r="D32" s="71"/>
+      <c r="E32" s="72"/>
+      <c r="F32" s="73"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="25"/>
+    </row>
+    <row r="33" spans="1:8" ht="16" thickBot="1">
+      <c r="A33" s="35"/>
+      <c r="B33" s="74"/>
+      <c r="C33" s="75"/>
+      <c r="D33" s="75"/>
+      <c r="E33" s="76"/>
+      <c r="F33" s="77"/>
+      <c r="G33" s="22"/>
+      <c r="H33" s="25"/>
+    </row>
+    <row r="34" spans="1:8" ht="30" customHeight="1">
+      <c r="A34" s="35"/>
+      <c r="B34" s="22"/>
+      <c r="C34" s="39" t="str">
+        <f>UPPER(C33)</f>
         <v/>
       </c>
-      <c r="D33" s="67"/>
-      <c r="E33" s="29"/>
-      <c r="F33" s="27"/>
-      <c r="G33" s="32"/>
-      <c r="H33" s="30"/>
-    </row>
-    <row r="34" spans="1:8">
-      <c r="A34" s="42"/>
-      <c r="B34" s="33"/>
-      <c r="C34" s="34"/>
-      <c r="D34" s="33"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="33"/>
-      <c r="G34" s="35"/>
-      <c r="H34" s="30"/>
+      <c r="D34" s="39"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="27"/>
+      <c r="H34" s="25"/>
     </row>
     <row r="35" spans="1:8">
-      <c r="H35" s="30"/>
+      <c r="A35" s="37"/>
+      <c r="B35" s="28"/>
+      <c r="C35" s="29"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="30"/>
+      <c r="H35" s="25"/>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="H36" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
     <mergeCell ref="C21:D21"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B30:F32"/>
-    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C23:D23"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="D5:F6"/>
     <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F33"/>
     <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="B29:F29"/>
   </mergeCells>
   <pageMargins left="0.9055118110236221" right="0.31496062992125984" top="0.74803149606299213" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="54" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>

</xml_diff>